<commit_message>
Add Tier 3 Full Universe tab — all 72 accounts named and segmented
3A: 14 active accounts (ACV > $0, score below 60) - content syndication
3B: 11 win-back priority (churned, significant LTV) - CSM win-back
3C: 47 awareness only (no active ACV) - product newsletter

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ABM-Playbooks/TinyMCE_AI_Upsell_Deal_Analysis.xlsx
+++ b/ABM-Playbooks/TinyMCE_AI_Upsell_Deal_Analysis.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Account List" sheetId="3" r:id="rId3"/>
     <sheet name="Lost Deals" sheetId="4" r:id="rId4"/>
     <sheet name="Scoring Summary" sheetId="5" r:id="rId5"/>
+    <sheet name="Tier 3 Full Universe" sheetId="6" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -3242,4 +3243,2208 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="30" customHeight="1"/>
+  <cols>
+    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t>Tier 3 - Full Account Universe (72 Accounts)</t>
+        </is>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr" s="10">
+        <is>
+          <t>SECTION 3A - ACTIVE CUSTOMERS (14 accounts, ACV &gt; 0, Priority Score below 60)</t>
+        </is>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="11">
+        <is>
+          <t>Account Name</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="11">
+        <is>
+          <t>Annual ACV</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="11">
+        <is>
+          <t>Lifetime ACV</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="11">
+        <is>
+          <t>App Category</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="11">
+        <is>
+          <t>TinyMCE Centrality</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="11">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="3">
+        <is>
+          <t>Exactera (Prev. CrossBorder Solutions)</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <v>24412</v>
+      </c>
+      <c r="C5" s="6">
+        <v>345372</v>
+      </c>
+      <c r="D5" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication + product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="3">
+        <is>
+          <t>Continu</t>
+        </is>
+      </c>
+      <c r="B6" s="6">
+        <v>27338</v>
+      </c>
+      <c r="C6" s="6">
+        <v>202543</v>
+      </c>
+      <c r="D6" t="inlineStr" s="3">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (EdTech)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="3">
+        <is>
+          <t>Eclectic IQ B.V.</t>
+        </is>
+      </c>
+      <c r="B7" s="6">
+        <v>11047</v>
+      </c>
+      <c r="C7" s="6">
+        <v>161267</v>
+      </c>
+      <c r="D7" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (cybersecurity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="3">
+        <is>
+          <t>ACGI Software</t>
+        </is>
+      </c>
+      <c r="B8" s="6">
+        <v>15362</v>
+      </c>
+      <c r="C8" s="6">
+        <v>182022</v>
+      </c>
+      <c r="D8" t="inlineStr" s="3">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication + product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="3">
+        <is>
+          <t>NAVEX Global (Previously Lockpath)</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <v>17556</v>
+      </c>
+      <c r="C9" s="6">
+        <v>127948</v>
+      </c>
+      <c r="D9" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (GRC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="3">
+        <is>
+          <t>LRN</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <v>21148</v>
+      </c>
+      <c r="C10" s="6">
+        <v>126886</v>
+      </c>
+      <c r="D10" t="inlineStr" s="3">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (compliance training)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="3">
+        <is>
+          <t>Catapult HQ</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <v>11550</v>
+      </c>
+      <c r="C11" s="6">
+        <v>126459</v>
+      </c>
+      <c r="D11" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="3">
+        <is>
+          <t>Manantial Ltd</t>
+        </is>
+      </c>
+      <c r="B12" s="6">
+        <v>18141</v>
+      </c>
+      <c r="C12" s="6">
+        <v>116567</v>
+      </c>
+      <c r="D12" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="3">
+        <is>
+          <t>InPhronesis LLC</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <v>12529</v>
+      </c>
+      <c r="C13" s="6">
+        <v>113313</v>
+      </c>
+      <c r="D13" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (pharma/life sciences)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="3">
+        <is>
+          <t>SOBIS Software GmbH</t>
+        </is>
+      </c>
+      <c r="B14" s="6">
+        <v>13145</v>
+      </c>
+      <c r="C14" s="6">
+        <v>96228</v>
+      </c>
+      <c r="D14" t="inlineStr" s="3">
+        <is>
+          <t>dms</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="3">
+        <is>
+          <t>Axero Holdings LLC</t>
+        </is>
+      </c>
+      <c r="B15" s="6">
+        <v>13379</v>
+      </c>
+      <c r="C15" s="6">
+        <v>72621</v>
+      </c>
+      <c r="D15" t="inlineStr" s="3">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication + product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="3">
+        <is>
+          <t>Axway Software SA (CYCOM Finances Groupe)</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <v>17303</v>
+      </c>
+      <c r="C16" s="6">
+        <v>71100</v>
+      </c>
+      <c r="D16" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr" s="3">
+        <is>
+          <t>Savills (UK) Limited</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <v>15675</v>
+      </c>
+      <c r="C17" s="6">
+        <v>55275</v>
+      </c>
+      <c r="D17" t="inlineStr" s="3">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="3">
+        <is>
+          <t>CourseAvenue</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <v>4194</v>
+      </c>
+      <c r="C18" s="6">
+        <v>25544</v>
+      </c>
+      <c r="D18" t="inlineStr" s="3">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="3">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="3">
+        <is>
+          <t>Content syndication (EdTech)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr" s="1">
+        <is>
+          <t>SECTION 3B - WIN-BACK PRIORITY (11 accounts, churned with significant Lifetime ACV)</t>
+        </is>
+      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr" s="11">
+        <is>
+          <t>Account Name</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="11">
+        <is>
+          <t>Annual ACV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="11">
+        <is>
+          <t>Lifetime ACV</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr" s="11">
+        <is>
+          <t>App Category</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr" s="11">
+        <is>
+          <t>TinyMCE Centrality</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr" s="11">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr" s="4">
+        <is>
+          <t>Moodle</t>
+        </is>
+      </c>
+      <c r="B22" s="7">
+        <v>0</v>
+      </c>
+      <c r="C22" s="7">
+        <v>3572800</v>
+      </c>
+      <c r="D22" t="inlineStr" s="4">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back + content syndication (LMS) - highest LTV on list</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr" s="4">
+        <is>
+          <t>Legislative Services Agency [CORPUS IN]</t>
+        </is>
+      </c>
+      <c r="B23" s="7">
+        <v>0</v>
+      </c>
+      <c r="C23" s="7">
+        <v>1271842</v>
+      </c>
+      <c r="D23" t="inlineStr" s="4">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - legislative workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr" s="4">
+        <is>
+          <t>Givebutter</t>
+        </is>
+      </c>
+      <c r="B24" s="7">
+        <v>0</v>
+      </c>
+      <c r="C24" s="7">
+        <v>826918</v>
+      </c>
+      <c r="D24" t="inlineStr" s="4">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - fundraising platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr" s="4">
+        <is>
+          <t>IP Copilot</t>
+        </is>
+      </c>
+      <c r="B25" s="7">
+        <v>0</v>
+      </c>
+      <c r="C25" s="7">
+        <v>519103</v>
+      </c>
+      <c r="D25" t="inlineStr" s="4">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - IP/patent drafting</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr" s="4">
+        <is>
+          <t>Microsoft [DragonMedicalOne and DaxCopilot]</t>
+        </is>
+      </c>
+      <c r="B26" s="7">
+        <v>0</v>
+      </c>
+      <c r="C26" s="7">
+        <v>446394</v>
+      </c>
+      <c r="D26" t="inlineStr" s="4">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr" s="4">
+        <is>
+          <t>Supporting</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - clinical AI workflow</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr" s="4">
+        <is>
+          <t>MIT Lincoln Laboratory</t>
+        </is>
+      </c>
+      <c r="B27" s="7">
+        <v>0</v>
+      </c>
+      <c r="C27" s="7">
+        <v>434820</v>
+      </c>
+      <c r="D27" t="inlineStr" s="4">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - government research</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr" s="4">
+        <is>
+          <t>Attentive Inc.</t>
+        </is>
+      </c>
+      <c r="B28" s="7">
+        <v>0</v>
+      </c>
+      <c r="C28" s="7">
+        <v>215828</v>
+      </c>
+      <c r="D28" t="inlineStr" s="4">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - sales automation OEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr" s="4">
+        <is>
+          <t>IBM [Tririga]</t>
+        </is>
+      </c>
+      <c r="B29" s="7">
+        <v>0</v>
+      </c>
+      <c r="C29" s="7">
+        <v>196367</v>
+      </c>
+      <c r="D29" t="inlineStr" s="4">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - facilities management</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr" s="4">
+        <is>
+          <t>Door Ventures</t>
+        </is>
+      </c>
+      <c r="B30" s="7">
+        <v>0</v>
+      </c>
+      <c r="C30" s="7">
+        <v>133897</v>
+      </c>
+      <c r="D30" t="inlineStr" s="4">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - fintech due diligence</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr" s="4">
+        <is>
+          <t>Campusknot</t>
+        </is>
+      </c>
+      <c r="B31" s="7">
+        <v>0</v>
+      </c>
+      <c r="C31" s="7">
+        <v>76200</v>
+      </c>
+      <c r="D31" t="inlineStr" s="4">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - higher ed engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr" s="4">
+        <is>
+          <t>Lone Wolf Technologies</t>
+        </is>
+      </c>
+      <c r="B32" s="7">
+        <v>0</v>
+      </c>
+      <c r="C32" s="7">
+        <v>65280</v>
+      </c>
+      <c r="D32" t="inlineStr" s="4">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr" s="4">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr" s="4">
+        <is>
+          <t>CSM win-back - real estate brokerage</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr" s="10">
+        <is>
+          <t>SECTION 3C - AWARENESS ONLY (47 accounts, no active ACV - product newsletter and content syndication only)</t>
+        </is>
+      </c>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr" s="11">
+        <is>
+          <t>Account Name</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr" s="11">
+        <is>
+          <t>Annual ACV</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="11">
+        <is>
+          <t>Lifetime ACV</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr" s="11">
+        <is>
+          <t>App Category</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr" s="11">
+        <is>
+          <t>TinyMCE Centrality</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr" s="11">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr" s="16">
+        <is>
+          <t>BNP Paribas [LOGO]</t>
+        </is>
+      </c>
+      <c r="B36" s="5">
+        <v>0</v>
+      </c>
+      <c r="C36" s="5">
+        <v>0</v>
+      </c>
+      <c r="D36" t="inlineStr" s="16">
+        <is>
+          <t>dms</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr" s="16">
+        <is>
+          <t>BloomAI</t>
+        </is>
+      </c>
+      <c r="B37" s="5">
+        <v>0</v>
+      </c>
+      <c r="C37" s="5">
+        <v>0</v>
+      </c>
+      <c r="D37" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr" s="16">
+        <is>
+          <t>CaseBlink</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <v>0</v>
+      </c>
+      <c r="C38" s="5">
+        <v>0</v>
+      </c>
+      <c r="D38" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr" s="16">
+        <is>
+          <t>Chase Software</t>
+        </is>
+      </c>
+      <c r="B39" s="5">
+        <v>0</v>
+      </c>
+      <c r="C39" s="5">
+        <v>0</v>
+      </c>
+      <c r="D39" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr" s="16">
+        <is>
+          <t>Cirrus Insight</t>
+        </is>
+      </c>
+      <c r="B40" s="5">
+        <v>0</v>
+      </c>
+      <c r="C40" s="5">
+        <v>0</v>
+      </c>
+      <c r="D40" t="inlineStr" s="16">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr" s="16">
+        <is>
+          <t>Cloud Driven Solutions</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <v>0</v>
+      </c>
+      <c r="C41" s="5">
+        <v>0</v>
+      </c>
+      <c r="D41" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr" s="16">
+        <is>
+          <t>Complaion</t>
+        </is>
+      </c>
+      <c r="B42" s="5">
+        <v>0</v>
+      </c>
+      <c r="C42" s="5">
+        <v>0</v>
+      </c>
+      <c r="D42" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (GRC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr" s="16">
+        <is>
+          <t>Craftly.AI</t>
+        </is>
+      </c>
+      <c r="B43" s="5">
+        <v>0</v>
+      </c>
+      <c r="C43" s="5">
+        <v>0</v>
+      </c>
+      <c r="D43" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr" s="16">
+        <is>
+          <t>Danaos Management Consultants S.A</t>
+        </is>
+      </c>
+      <c r="B44" s="5">
+        <v>0</v>
+      </c>
+      <c r="C44" s="5">
+        <v>0</v>
+      </c>
+      <c r="D44" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr" s="16">
+        <is>
+          <t>Deposyt</t>
+        </is>
+      </c>
+      <c r="B45" s="5">
+        <v>0</v>
+      </c>
+      <c r="C45" s="5">
+        <v>0</v>
+      </c>
+      <c r="D45" t="inlineStr" s="16">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr" s="16">
+        <is>
+          <t>Gallium</t>
+        </is>
+      </c>
+      <c r="B46" s="5">
+        <v>0</v>
+      </c>
+      <c r="C46" s="5">
+        <v>0</v>
+      </c>
+      <c r="D46" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr" s="16">
+        <is>
+          <t>Graphite</t>
+        </is>
+      </c>
+      <c r="B47" s="5">
+        <v>0</v>
+      </c>
+      <c r="C47" s="5">
+        <v>0</v>
+      </c>
+      <c r="D47" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr" s="16">
+        <is>
+          <t>Hazel AI Technologies</t>
+        </is>
+      </c>
+      <c r="B48" s="5">
+        <v>0</v>
+      </c>
+      <c r="C48" s="5">
+        <v>0</v>
+      </c>
+      <c r="D48" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr" s="16">
+        <is>
+          <t>Helsana Insurance Company Ltd</t>
+        </is>
+      </c>
+      <c r="B49" s="5">
+        <v>0</v>
+      </c>
+      <c r="C49" s="5">
+        <v>0</v>
+      </c>
+      <c r="D49" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr" s="16">
+        <is>
+          <t>ISMS Applications</t>
+        </is>
+      </c>
+      <c r="B50" s="5">
+        <v>0</v>
+      </c>
+      <c r="C50" s="5">
+        <v>0</v>
+      </c>
+      <c r="D50" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (GRC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr" s="16">
+        <is>
+          <t>Jobflow</t>
+        </is>
+      </c>
+      <c r="B51" s="5">
+        <v>0</v>
+      </c>
+      <c r="C51" s="5">
+        <v>0</v>
+      </c>
+      <c r="D51" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr" s="16">
+        <is>
+          <t>Kaiso</t>
+        </is>
+      </c>
+      <c r="B52" s="5">
+        <v>0</v>
+      </c>
+      <c r="C52" s="5">
+        <v>0</v>
+      </c>
+      <c r="D52" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (GRC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr" s="16">
+        <is>
+          <t>Keyzo</t>
+        </is>
+      </c>
+      <c r="B53" s="5">
+        <v>0</v>
+      </c>
+      <c r="C53" s="5">
+        <v>0</v>
+      </c>
+      <c r="D53" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr" s="16">
+        <is>
+          <t>Knowt</t>
+        </is>
+      </c>
+      <c r="B54" s="5">
+        <v>0</v>
+      </c>
+      <c r="C54" s="5">
+        <v>0</v>
+      </c>
+      <c r="D54" t="inlineStr" s="16">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (EdTech)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr" s="16">
+        <is>
+          <t>Laud.Ai</t>
+        </is>
+      </c>
+      <c r="B55" s="5">
+        <v>0</v>
+      </c>
+      <c r="C55" s="5">
+        <v>0</v>
+      </c>
+      <c r="D55" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr" s="16">
+        <is>
+          <t>Legend Web Works</t>
+        </is>
+      </c>
+      <c r="B56" s="5">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5">
+        <v>0</v>
+      </c>
+      <c r="D56" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr" s="16">
+        <is>
+          <t>MaxCredible</t>
+        </is>
+      </c>
+      <c r="B57" s="5">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5">
+        <v>0</v>
+      </c>
+      <c r="D57" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr" s="16">
+        <is>
+          <t>MIT Lincoln Laboratory</t>
+        </is>
+      </c>
+      <c r="B58" s="5">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5">
+        <v>0</v>
+      </c>
+      <c r="D58" t="inlineStr" s="16">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr" s="16">
+        <is>
+          <t>Naverisk</t>
+        </is>
+      </c>
+      <c r="B59" s="5">
+        <v>0</v>
+      </c>
+      <c r="C59" s="5">
+        <v>0</v>
+      </c>
+      <c r="D59" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr" s="16">
+        <is>
+          <t>Netpresenter BV</t>
+        </is>
+      </c>
+      <c r="B60" s="5">
+        <v>0</v>
+      </c>
+      <c r="C60" s="5">
+        <v>0</v>
+      </c>
+      <c r="D60" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr" s="16">
+        <is>
+          <t>OIM Consulting (Pty) Ltd.</t>
+        </is>
+      </c>
+      <c r="B61" s="5">
+        <v>0</v>
+      </c>
+      <c r="C61" s="5">
+        <v>0</v>
+      </c>
+      <c r="D61" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr" s="16">
+        <is>
+          <t>One To One Plus</t>
+        </is>
+      </c>
+      <c r="B62" s="5">
+        <v>0</v>
+      </c>
+      <c r="C62" s="5">
+        <v>0</v>
+      </c>
+      <c r="D62" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr" s="16">
+        <is>
+          <t>Panodyssey</t>
+        </is>
+      </c>
+      <c r="B63" s="5">
+        <v>0</v>
+      </c>
+      <c r="C63" s="5">
+        <v>0</v>
+      </c>
+      <c r="D63" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr" s="16">
+        <is>
+          <t>PhaseZero.ai</t>
+        </is>
+      </c>
+      <c r="B64" s="5">
+        <v>0</v>
+      </c>
+      <c r="C64" s="5">
+        <v>0</v>
+      </c>
+      <c r="D64" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr" s="16">
+        <is>
+          <t>Plexus.co</t>
+        </is>
+      </c>
+      <c r="B65" s="5">
+        <v>0</v>
+      </c>
+      <c r="C65" s="5">
+        <v>0</v>
+      </c>
+      <c r="D65" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr" s="16">
+        <is>
+          <t>Prodeology</t>
+        </is>
+      </c>
+      <c r="B66" s="5">
+        <v>0</v>
+      </c>
+      <c r="C66" s="5">
+        <v>0</v>
+      </c>
+      <c r="D66" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr" s="16">
+        <is>
+          <t>Prodlane GmbH</t>
+        </is>
+      </c>
+      <c r="B67" s="5">
+        <v>0</v>
+      </c>
+      <c r="C67" s="5">
+        <v>0</v>
+      </c>
+      <c r="D67" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr" s="16">
+        <is>
+          <t>Precis AI</t>
+        </is>
+      </c>
+      <c r="B68" s="5">
+        <v>0</v>
+      </c>
+      <c r="C68" s="5">
+        <v>0</v>
+      </c>
+      <c r="D68" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr" s="16">
+        <is>
+          <t>Shoper S.A.</t>
+        </is>
+      </c>
+      <c r="B69" s="5">
+        <v>0</v>
+      </c>
+      <c r="C69" s="5">
+        <v>0</v>
+      </c>
+      <c r="D69" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr" s="16">
+        <is>
+          <t>Soxhub</t>
+        </is>
+      </c>
+      <c r="B70" s="5">
+        <v>0</v>
+      </c>
+      <c r="C70" s="5">
+        <v>0</v>
+      </c>
+      <c r="D70" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (GRC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr" s="16">
+        <is>
+          <t>Teachmint</t>
+        </is>
+      </c>
+      <c r="B71" s="5">
+        <v>0</v>
+      </c>
+      <c r="C71" s="5">
+        <v>0</v>
+      </c>
+      <c r="D71" t="inlineStr" s="16">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (EdTech)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr" s="16">
+        <is>
+          <t>TestU Labs</t>
+        </is>
+      </c>
+      <c r="B72" s="5">
+        <v>0</v>
+      </c>
+      <c r="C72" s="5">
+        <v>0</v>
+      </c>
+      <c r="D72" t="inlineStr" s="16">
+        <is>
+          <t>lms</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter + content syndication (EdTech)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr" s="16">
+        <is>
+          <t>TownSquare</t>
+        </is>
+      </c>
+      <c r="B73" s="5">
+        <v>0</v>
+      </c>
+      <c r="C73" s="5">
+        <v>0</v>
+      </c>
+      <c r="D73" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr" s="16">
+        <is>
+          <t>UTF</t>
+        </is>
+      </c>
+      <c r="B74" s="5">
+        <v>0</v>
+      </c>
+      <c r="C74" s="5">
+        <v>0</v>
+      </c>
+      <c r="D74" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr" s="16">
+        <is>
+          <t>Urbanise</t>
+        </is>
+      </c>
+      <c r="B75" s="5">
+        <v>0</v>
+      </c>
+      <c r="C75" s="5">
+        <v>0</v>
+      </c>
+      <c r="D75" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr" s="16">
+        <is>
+          <t>V2K AI</t>
+        </is>
+      </c>
+      <c r="B76" s="5">
+        <v>0</v>
+      </c>
+      <c r="C76" s="5">
+        <v>0</v>
+      </c>
+      <c r="D76" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr" s="16">
+        <is>
+          <t>Veriday</t>
+        </is>
+      </c>
+      <c r="B77" s="5">
+        <v>0</v>
+      </c>
+      <c r="C77" s="5">
+        <v>0</v>
+      </c>
+      <c r="D77" t="inlineStr" s="16">
+        <is>
+          <t>cms</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr" s="16">
+        <is>
+          <t>WAFIOS AG</t>
+        </is>
+      </c>
+      <c r="B78" s="5">
+        <v>0</v>
+      </c>
+      <c r="C78" s="5">
+        <v>0</v>
+      </c>
+      <c r="D78" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr" s="16">
+        <is>
+          <t>Witivio</t>
+        </is>
+      </c>
+      <c r="B79" s="5">
+        <v>0</v>
+      </c>
+      <c r="C79" s="5">
+        <v>0</v>
+      </c>
+      <c r="D79" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr" s="16">
+        <is>
+          <t>gpac</t>
+        </is>
+      </c>
+      <c r="B80" s="5">
+        <v>0</v>
+      </c>
+      <c r="C80" s="5">
+        <v>0</v>
+      </c>
+      <c r="D80" t="inlineStr" s="16">
+        <is>
+          <t>crm</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr" s="16">
+        <is>
+          <t>iTacit</t>
+        </is>
+      </c>
+      <c r="B81" s="5">
+        <v>0</v>
+      </c>
+      <c r="C81" s="5">
+        <v>0</v>
+      </c>
+      <c r="D81" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr" s="16">
+        <is>
+          <t>neoshare AG</t>
+        </is>
+      </c>
+      <c r="B82" s="5">
+        <v>0</v>
+      </c>
+      <c r="C82" s="5">
+        <v>0</v>
+      </c>
+      <c r="D82" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr" s="16">
+        <is>
+          <t>vip district</t>
+        </is>
+      </c>
+      <c r="B83" s="5">
+        <v>0</v>
+      </c>
+      <c r="C83" s="5">
+        <v>0</v>
+      </c>
+      <c r="D83" t="inlineStr" s="16">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr" s="16">
+        <is>
+          <t>Core</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr" s="16">
+        <is>
+          <t>Product newsletter</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>